<commit_message>
Null-calibrated interaction information, Figure 1c (additivity), composite Figure 1
- R5_reviewer_checks/run_interaction_calibration.py: within-class shuffling null per LOCO
  fold; super-additive consensus pairs 14.8 % (taxa), 10.0 % (functions), 8.1 % (combined);
  42 of 235 stable pairs; columns added to Supp. Tables 2 and 4
- R1 figure1b_all_pairs/plot_figure1c_additivity.py: total IG vs sum of individual IGs
- manuscript/make_figure1.py: Figure 1 = schematic + b (directional) + c (additivity)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manuscript/supplementary/Supplementary_tables.xlsx
+++ b/manuscript/supplementary/Supplementary_tables.xlsx
@@ -1398,7 +1398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1409,12 +1409,15 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="90" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Supplementary Table 2. The 30 directed synergistic feature pairs with the highest mean total 2D information gain (IG) across the taxa-only, functions-only and combined analyses. base_IG_1D_mean: 1D IG of the base feature; total_IG_2D_mean: joint IG of the pair (base 1D IG + IG added by the contributing feature); ig_difference_raw / ig_difference_pct: absolute and relative gain over the base feature; pair_ig_count: number of fold-run combinations (of 140 = 14 LOCO folds x 10 MDFS runs) in which the pair was among the top 2 % of pairs.</t>
+          <t>Supplementary Table 2. The 30 directed synergistic feature pairs with the highest mean total 2D information gain (IG) across the taxa-only, functions-only and combined analyses. base_IG_1D_mean: 1D IG of the base feature; total_IG_2D_mean: joint IG of the pair (base 1D IG + IG added by the contributing feature); ig_difference_raw / ig_difference_pct: absolute and relative gain over the base feature; pair_ig_count: number of fold-run combinations (of 140 = 14 LOCO folds x 10 MDFS runs) in which the pair was among the top 2 % of pairs. interaction_information_mean: total IG of the pair minus the two individual IGs, averaged over the fold-runs in which the pair was selected; pct_fold_runs_super_additive: share of those fold-runs in which it exceeded the chance threshold obtained by within-class shuffling of the features; super_additive: that share is at least 50 %.</t>
         </is>
       </c>
     </row>
@@ -1459,6 +1462,21 @@
           <t>pair_ig_count</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>interaction_information_mean</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>pct_fold_runs_super_additive</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>super_additive</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1493,6 +1511,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I4" t="n">
+        <v>-193.65</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1527,6 +1556,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I5" t="n">
+        <v>-193.65</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1561,6 +1601,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I6" t="n">
+        <v>-192.81</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1595,6 +1646,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I7" t="n">
+        <v>-192.81</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1629,6 +1691,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I8" t="n">
+        <v>-214.06</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1663,6 +1736,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I9" t="n">
+        <v>-214.06</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1697,6 +1781,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I10" t="n">
+        <v>-214.03</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1731,6 +1826,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I11" t="n">
+        <v>-214.03</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1765,6 +1871,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I12" t="n">
+        <v>-196.5</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1799,6 +1916,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I13" t="n">
+        <v>-196.5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1833,6 +1961,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I14" t="n">
+        <v>-189.78</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1867,6 +2006,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I15" t="n">
+        <v>-189.78</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1901,6 +2051,17 @@
           <t>134/140</t>
         </is>
       </c>
+      <c r="I16" t="n">
+        <v>-76.81999999999999</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1935,6 +2096,17 @@
           <t>134/140</t>
         </is>
       </c>
+      <c r="I17" t="n">
+        <v>-76.81999999999999</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1969,6 +2141,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I18" t="n">
+        <v>-76.77</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2003,6 +2186,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I19" t="n">
+        <v>-76.77</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2037,6 +2231,17 @@
           <t>138/140</t>
         </is>
       </c>
+      <c r="I20" t="n">
+        <v>-180.26</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2071,6 +2276,17 @@
           <t>138/140</t>
         </is>
       </c>
+      <c r="I21" t="n">
+        <v>-180.26</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2105,6 +2321,17 @@
           <t>9/140</t>
         </is>
       </c>
+      <c r="I22" t="n">
+        <v>-32.85</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2139,6 +2366,17 @@
           <t>9/140</t>
         </is>
       </c>
+      <c r="I23" t="n">
+        <v>-32.85</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2173,6 +2411,17 @@
           <t>10/140</t>
         </is>
       </c>
+      <c r="I24" t="n">
+        <v>-32.08</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2207,6 +2456,17 @@
           <t>10/140</t>
         </is>
       </c>
+      <c r="I25" t="n">
+        <v>-32.08</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2241,6 +2501,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I26" t="n">
+        <v>-177.73</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2275,6 +2546,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I27" t="n">
+        <v>-177.73</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2309,6 +2591,17 @@
           <t>134/140</t>
         </is>
       </c>
+      <c r="I28" t="n">
+        <v>-166.5</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2343,6 +2636,17 @@
           <t>134/140</t>
         </is>
       </c>
+      <c r="I29" t="n">
+        <v>-166.5</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2377,6 +2681,17 @@
           <t>9/140</t>
         </is>
       </c>
+      <c r="I30" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2411,6 +2726,17 @@
           <t>9/140</t>
         </is>
       </c>
+      <c r="I31" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2445,6 +2771,17 @@
           <t>140/140</t>
         </is>
       </c>
+      <c r="I32" t="n">
+        <v>-165.6</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2477,6 +2814,17 @@
       <c r="H33" t="inlineStr">
         <is>
           <t>140/140</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>-165.6</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -2885,7 +3233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M238"/>
+  <dimension ref="A1:P238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2901,12 +3249,15 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="90" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Supplementary Table 4. Stable synthetic feature pairs in the CRC data: pairs whose synthetic feature was selected by the final random forest in &gt;= 80 % of the 14 LOCO folds and more often than either constituent (Selection % Gain = pair frequency minus the mean frequency of its constituents). Post-selection effect-size summary per pair: transformation evaluated in most cohorts, number of two-class cohorts, Benjamini-Hochberg q of the Stouffer meta p-value across cohorts, median rank-biserial correlation (positive = higher in CRC) and the number of cohorts with positive / negative direction.</t>
+          <t>Supplementary Table 4. Stable synthetic feature pairs in the CRC data: pairs whose synthetic feature was selected by the final random forest in &gt;= 80 % of the 14 LOCO folds and more often than either constituent (Selection % Gain = pair frequency minus the mean frequency of its constituents). Post-selection effect-size summary per pair: transformation evaluated in most cohorts, number of two-class cohorts, Benjamini-Hochberg q of the Stouffer meta p-value across cohorts, median rank-biserial correlation (positive = higher in CRC) and the number of cohorts with positive / negative direction. interaction_information_mean: total IG of the pair minus the two individual IGs, averaged over the fold-runs in which the pair was selected; pct_fold_runs_super_additive: share of those fold-runs in which it exceeded the chance threshold obtained by within-class shuffling of the features; super_additive: that share is at least 50 %.</t>
         </is>
       </c>
     </row>
@@ -2976,6 +3327,21 @@
           <t>Direction (+CRC/-CRC)</t>
         </is>
       </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>interaction_information_mean</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>pct_fold_runs_super_additive</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>super_additive</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3027,6 +3393,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N4" t="n">
+        <v>26.68</v>
+      </c>
+      <c r="O4" t="n">
+        <v>100</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3078,6 +3455,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N5" t="n">
+        <v>-36.4</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3129,6 +3517,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N6" t="n">
+        <v>-177.48</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3180,6 +3579,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N7" t="n">
+        <v>-220.18</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3231,6 +3641,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N8" t="n">
+        <v>-177.73</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3282,6 +3703,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N9" t="n">
+        <v>-19.08</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3333,6 +3765,17 @@
           <t>+2/-13</t>
         </is>
       </c>
+      <c r="N10" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3374,7 +3817,7 @@
         <v>15</v>
       </c>
       <c r="K11" t="n">
-        <v>1.761188411635734e-41</v>
+        <v>1.761188411635733e-41</v>
       </c>
       <c r="L11" t="n">
         <v>-0.4112615823235923</v>
@@ -3384,6 +3827,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N11" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="O11" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3435,6 +3889,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N12" t="n">
+        <v>18.09</v>
+      </c>
+      <c r="O12" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3486,6 +3951,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N13" t="n">
+        <v>-17.24</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3537,6 +4013,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N14" t="n">
+        <v>-28.38</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3588,6 +4075,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N15" t="n">
+        <v>-193.65</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3639,6 +4137,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N16" t="n">
+        <v>-57.45</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3690,6 +4199,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N17" t="n">
+        <v>-20.07</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3741,6 +4261,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N18" t="n">
+        <v>-11.33</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3792,6 +4323,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N19" t="n">
+        <v>-53.27</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3843,6 +4385,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N20" t="n">
+        <v>-12.31</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3894,6 +4447,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N21" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="O21" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3945,6 +4509,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N22" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="O22" t="n">
+        <v>100</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3996,6 +4571,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N23" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="O23" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4047,6 +4633,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N24" t="n">
+        <v>-50.51</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4098,6 +4695,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N25" t="n">
+        <v>-165.6</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4149,6 +4757,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N26" t="n">
+        <v>-214.06</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4200,6 +4819,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N27" t="n">
+        <v>-196.5</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4251,6 +4881,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N28" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4302,6 +4943,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N29" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="O29" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4353,6 +5005,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N30" t="n">
+        <v>13.48</v>
+      </c>
+      <c r="O30" t="n">
+        <v>97.73999999999999</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4404,6 +5067,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N31" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4455,6 +5129,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N32" t="n">
+        <v>-50.07</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4506,6 +5191,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N33" t="n">
+        <v>-7.33</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4557,6 +5253,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N34" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4608,6 +5315,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N35" t="n">
+        <v>-38.42</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4659,6 +5377,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N36" t="n">
+        <v>-4.94</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4710,6 +5439,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N37" t="n">
+        <v>-10.03</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4761,6 +5501,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N38" t="n">
+        <v>-1.21</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4812,6 +5563,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N39" t="n">
+        <v>-37.47</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4863,6 +5625,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N40" t="n">
+        <v>-8.42</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4914,6 +5687,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N41" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="O41" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4965,6 +5749,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N42" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5016,6 +5811,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N43" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5067,6 +5873,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N44" t="n">
+        <v>-13.59</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5118,6 +5935,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N45" t="n">
+        <v>-10.48</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5169,6 +5997,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N46" t="n">
+        <v>-16.01</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5220,6 +6059,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N47" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5271,6 +6121,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N48" t="n">
+        <v>-2.58</v>
+      </c>
+      <c r="O48" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5322,6 +6183,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N49" t="n">
+        <v>-42.19</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5373,6 +6245,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N50" t="n">
+        <v>-10.57</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5424,6 +6307,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N51" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="O51" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5475,6 +6369,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N52" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5526,6 +6431,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N53" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5577,6 +6493,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N54" t="n">
+        <v>-5.02</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5628,6 +6555,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N55" t="n">
+        <v>-10.53</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5679,6 +6617,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N56" t="n">
+        <v>-10.18</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5730,6 +6679,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N57" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="O57" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5771,7 +6731,7 @@
         <v>15</v>
       </c>
       <c r="K58" t="n">
-        <v>4.406298448788378e-44</v>
+        <v>4.406298448788379e-44</v>
       </c>
       <c r="L58" t="n">
         <v>0.3879882092851878</v>
@@ -5781,6 +6741,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N58" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="O58" t="n">
+        <v>87.22</v>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5832,6 +6803,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N59" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="O59" t="n">
+        <v>93.23</v>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5883,6 +6865,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N60" t="n">
+        <v>-30.83</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5934,6 +6927,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N61" t="n">
+        <v>-63.99</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5985,6 +6989,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N62" t="n">
+        <v>-72.54000000000001</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6036,6 +7051,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N63" t="n">
+        <v>-58.67</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6087,6 +7113,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N64" t="n">
+        <v>-7.64</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -6138,6 +7175,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N65" t="n">
+        <v>16.53</v>
+      </c>
+      <c r="O65" t="n">
+        <v>97.73999999999999</v>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6189,6 +7237,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N66" t="n">
+        <v>-76.77</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6240,6 +7299,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N67" t="n">
+        <v>22.98</v>
+      </c>
+      <c r="O67" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6291,6 +7361,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N68" t="n">
+        <v>23.02</v>
+      </c>
+      <c r="O68" t="n">
+        <v>97.01000000000001</v>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6342,6 +7423,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N69" t="n">
+        <v>-10.28</v>
+      </c>
+      <c r="O69" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6393,6 +7485,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N70" t="n">
+        <v>29.02</v>
+      </c>
+      <c r="O70" t="n">
+        <v>100</v>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6444,6 +7547,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N71" t="n">
+        <v>19.74</v>
+      </c>
+      <c r="O71" t="n">
+        <v>100</v>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6495,6 +7609,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N72" t="n">
+        <v>-15.52</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6546,6 +7671,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N73" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="O73" t="n">
+        <v>89.47</v>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6597,6 +7733,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N74" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="O74" t="n">
+        <v>97.73999999999999</v>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6648,6 +7795,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N75" t="n">
+        <v>-9.380000000000001</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6699,6 +7857,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N76" t="n">
+        <v>-17.75</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0</v>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6750,6 +7919,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N77" t="n">
+        <v>-20.79</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0</v>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6801,6 +7981,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N78" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0</v>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6852,6 +8043,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N79" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="O79" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6903,6 +8105,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N80" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="O80" t="n">
+        <v>30.53</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6954,6 +8167,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N81" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O81" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7005,6 +8229,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N82" t="n">
+        <v>-12.49</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7056,6 +8291,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N83" t="n">
+        <v>-8.26</v>
+      </c>
+      <c r="O83" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7107,6 +8353,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N84" t="n">
+        <v>-9.210000000000001</v>
+      </c>
+      <c r="O84" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7158,6 +8415,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N85" t="n">
+        <v>-9.92</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0</v>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7209,6 +8477,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N86" t="n">
+        <v>-21.43</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0</v>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7260,6 +8539,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N87" t="n">
+        <v>-8.27</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0</v>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7311,6 +8601,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N88" t="n">
+        <v>-3.91</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7362,6 +8663,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N89" t="n">
+        <v>-40.3</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0</v>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7413,6 +8725,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N90" t="n">
+        <v>-12.24</v>
+      </c>
+      <c r="O90" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7464,6 +8787,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N91" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7515,6 +8849,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N92" t="n">
+        <v>-11.58</v>
+      </c>
+      <c r="O92" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7566,6 +8911,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N93" t="n">
+        <v>-14.48</v>
+      </c>
+      <c r="O93" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7617,6 +8973,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N94" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7668,6 +9035,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N95" t="n">
+        <v>-18.64</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7719,6 +9097,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N96" t="n">
+        <v>-2.38</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7770,6 +9159,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N97" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="O97" t="n">
+        <v>13.53</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7821,6 +9221,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N98" t="n">
+        <v>-11.12</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0</v>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7872,6 +9283,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N99" t="n">
+        <v>-9.359999999999999</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0</v>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7923,6 +9345,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N100" t="n">
+        <v>-7.23</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0</v>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7974,6 +9407,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N101" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="O101" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8015,7 +9459,7 @@
         <v>15</v>
       </c>
       <c r="K102" t="n">
-        <v>4.037055400489961e-66</v>
+        <v>4.037055400489962e-66</v>
       </c>
       <c r="L102" t="n">
         <v>-0.4868778280542987</v>
@@ -8025,6 +9469,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N102" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0</v>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8076,6 +9531,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N103" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0</v>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8127,6 +9593,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N104" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="O104" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8178,6 +9655,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N105" t="n">
+        <v>-4.21</v>
+      </c>
+      <c r="O105" t="n">
+        <v>0</v>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8229,6 +9717,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N106" t="n">
+        <v>-3.15</v>
+      </c>
+      <c r="O106" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8280,6 +9779,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N107" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="O107" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8331,6 +9841,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N108" t="n">
+        <v>-2.48</v>
+      </c>
+      <c r="O108" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8382,6 +9903,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N109" t="n">
+        <v>-25.23</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -8423,7 +9955,7 @@
         <v>15</v>
       </c>
       <c r="K110" t="n">
-        <v>7.351197390495679e-55</v>
+        <v>7.351197390495678e-55</v>
       </c>
       <c r="L110" t="n">
         <v>0.4608753315649867</v>
@@ -8433,6 +9965,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N110" t="n">
+        <v>-6.89</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8484,6 +10027,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N111" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0</v>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8535,6 +10089,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N112" t="n">
+        <v>-1.29</v>
+      </c>
+      <c r="O112" t="n">
+        <v>0</v>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8586,6 +10151,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N113" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="O113" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8637,6 +10213,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N114" t="n">
+        <v>-4.62</v>
+      </c>
+      <c r="O114" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8688,6 +10275,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N115" t="n">
+        <v>-0.73</v>
+      </c>
+      <c r="O115" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8739,6 +10337,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N116" t="n">
+        <v>-9.35</v>
+      </c>
+      <c r="O116" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8790,6 +10399,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N117" t="n">
+        <v>-3.74</v>
+      </c>
+      <c r="O117" t="n">
+        <v>0</v>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8841,6 +10461,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N118" t="n">
+        <v>-4.08</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0</v>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8892,6 +10523,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N119" t="n">
+        <v>-24.5</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0</v>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8943,6 +10585,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N120" t="n">
+        <v>-20.33</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0</v>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8994,6 +10647,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N121" t="n">
+        <v>-9.4</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -9045,6 +10709,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N122" t="n">
+        <v>-18.62</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0</v>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -9096,6 +10771,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N123" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="O123" t="n">
+        <v>100</v>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -9147,6 +10833,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N124" t="n">
+        <v>-3.39</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -9198,6 +10895,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N125" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="O125" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9249,6 +10957,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N126" t="n">
+        <v>-6.75</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9300,6 +11019,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N127" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="O127" t="n">
+        <v>100</v>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -9341,7 +11071,7 @@
         <v>15</v>
       </c>
       <c r="K128" t="n">
-        <v>1.556814462631828e-55</v>
+        <v>1.556814462631827e-55</v>
       </c>
       <c r="L128" t="n">
         <v>0.2838</v>
@@ -9351,6 +11081,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N128" t="n">
+        <v>-25.93</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0</v>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9402,6 +11143,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N129" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="O129" t="n">
+        <v>0</v>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9453,6 +11205,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N130" t="n">
+        <v>-25.23</v>
+      </c>
+      <c r="O130" t="n">
+        <v>0</v>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9504,6 +11267,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N131" t="n">
+        <v>-8.27</v>
+      </c>
+      <c r="O131" t="n">
+        <v>0</v>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9555,6 +11329,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N132" t="n">
+        <v>-6.27</v>
+      </c>
+      <c r="O132" t="n">
+        <v>0</v>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9606,6 +11391,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N133" t="n">
+        <v>-7.55</v>
+      </c>
+      <c r="O133" t="n">
+        <v>0</v>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9657,6 +11453,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N134" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="O134" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9708,6 +11515,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N135" t="n">
+        <v>-18.22</v>
+      </c>
+      <c r="O135" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9759,6 +11577,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N136" t="n">
+        <v>-7.34</v>
+      </c>
+      <c r="O136" t="n">
+        <v>0</v>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9810,6 +11639,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N137" t="n">
+        <v>-8.91</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9861,6 +11701,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N138" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O138" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9912,6 +11763,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N139" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="O139" t="n">
+        <v>0</v>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9963,6 +11825,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N140" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="O140" t="n">
+        <v>0</v>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -10014,6 +11887,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N141" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -10065,6 +11949,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N142" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="O142" t="n">
+        <v>37.59</v>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -10116,6 +12011,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N143" t="n">
+        <v>-4.64</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -10167,6 +12073,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N144" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="O144" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -10218,6 +12135,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N145" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="O145" t="n">
+        <v>0</v>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10269,6 +12197,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N146" t="n">
+        <v>-8.640000000000001</v>
+      </c>
+      <c r="O146" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10310,7 +12249,7 @@
         <v>15</v>
       </c>
       <c r="K147" t="n">
-        <v>6.170586090138004e-54</v>
+        <v>6.170586090138003e-54</v>
       </c>
       <c r="L147" t="n">
         <v>0.5800000000000001</v>
@@ -10320,6 +12259,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N147" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="O147" t="n">
+        <v>29.01</v>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10371,6 +12321,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N148" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="O148" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10422,6 +12383,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N149" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="O149" t="n">
+        <v>7.52</v>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10473,6 +12445,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N150" t="n">
+        <v>-8.710000000000001</v>
+      </c>
+      <c r="O150" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10524,6 +12507,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N151" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="O151" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10575,6 +12569,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N152" t="n">
+        <v>-6.31</v>
+      </c>
+      <c r="O152" t="n">
+        <v>0</v>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10626,6 +12631,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N153" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="O153" t="n">
+        <v>86.47</v>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -10677,6 +12693,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N154" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="O154" t="n">
+        <v>53.38</v>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -10728,6 +12755,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N155" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0</v>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -10779,6 +12817,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N156" t="n">
+        <v>-11.2</v>
+      </c>
+      <c r="O156" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10830,6 +12879,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N157" t="n">
+        <v>-17.36</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0</v>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10881,6 +12941,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N158" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0</v>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -10932,6 +13003,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N159" t="n">
+        <v>-9.640000000000001</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0</v>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -10983,6 +13065,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N160" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="O160" t="n">
+        <v>0</v>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -11034,6 +13127,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N161" t="n">
+        <v>-11.41</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0</v>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11085,6 +13189,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N162" t="n">
+        <v>-33.34</v>
+      </c>
+      <c r="O162" t="n">
+        <v>0</v>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11136,6 +13251,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N163" t="n">
+        <v>-11.76</v>
+      </c>
+      <c r="O163" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11187,6 +13313,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N164" t="n">
+        <v>7.64</v>
+      </c>
+      <c r="O164" t="n">
+        <v>75.19</v>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11238,6 +13375,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N165" t="n">
+        <v>-3.74</v>
+      </c>
+      <c r="O165" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11289,6 +13437,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N166" t="n">
+        <v>-27.17</v>
+      </c>
+      <c r="O166" t="n">
+        <v>0</v>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11340,6 +13499,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N167" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="O167" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11391,6 +13561,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N168" t="n">
+        <v>-16.34</v>
+      </c>
+      <c r="O168" t="n">
+        <v>0</v>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11442,6 +13623,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N169" t="n">
+        <v>-4.73</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0</v>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -11493,6 +13685,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N170" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0</v>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -11544,6 +13747,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N171" t="n">
+        <v>-16.06</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -11595,6 +13809,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N172" t="n">
+        <v>-18.85</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0</v>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -11646,6 +13871,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N173" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="O173" t="n">
+        <v>17.83</v>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -11697,6 +13933,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N174" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="O174" t="n">
+        <v>100</v>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -11748,6 +13995,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N175" t="n">
+        <v>-40.88</v>
+      </c>
+      <c r="O175" t="n">
+        <v>0</v>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -11799,6 +14057,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N176" t="n">
+        <v>-6.63</v>
+      </c>
+      <c r="O176" t="n">
+        <v>0</v>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -11850,6 +14119,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N177" t="n">
+        <v>-42.07</v>
+      </c>
+      <c r="O177" t="n">
+        <v>0</v>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -11901,6 +14181,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N178" t="n">
+        <v>-3.19</v>
+      </c>
+      <c r="O178" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -11952,6 +14243,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N179" t="n">
+        <v>-30.75</v>
+      </c>
+      <c r="O179" t="n">
+        <v>0</v>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -11993,7 +14295,7 @@
         <v>15</v>
       </c>
       <c r="K180" t="n">
-        <v>4.476733763808068e-10</v>
+        <v>4.476733763808067e-10</v>
       </c>
       <c r="L180" t="n">
         <v>0.1740064446831364</v>
@@ -12003,6 +14305,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N180" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="O180" t="n">
+        <v>0</v>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12054,6 +14367,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N181" t="n">
+        <v>-9.119999999999999</v>
+      </c>
+      <c r="O181" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12105,6 +14429,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N182" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="O182" t="n">
+        <v>54.81</v>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12156,6 +14491,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N183" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="O183" t="n">
+        <v>98.25</v>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12207,6 +14553,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N184" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="O184" t="n">
+        <v>92.66</v>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -12258,6 +14615,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N185" t="n">
+        <v>17.11</v>
+      </c>
+      <c r="O185" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -12309,6 +14677,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N186" t="n">
+        <v>-19.11</v>
+      </c>
+      <c r="O186" t="n">
+        <v>0</v>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -12360,6 +14739,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N187" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="O187" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -12411,6 +14801,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N188" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="O188" t="n">
+        <v>94.06</v>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -12462,6 +14863,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N189" t="n">
+        <v>-4.07</v>
+      </c>
+      <c r="O189" t="n">
+        <v>0</v>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -12513,6 +14925,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N190" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="O190" t="n">
+        <v>85.58</v>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -12564,6 +14987,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N191" t="n">
+        <v>17.35</v>
+      </c>
+      <c r="O191" t="n">
+        <v>100</v>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -12615,6 +15049,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N192" t="n">
+        <v>-33.41</v>
+      </c>
+      <c r="O192" t="n">
+        <v>0</v>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -12666,6 +15111,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N193" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="O193" t="n">
+        <v>97.98</v>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -12717,6 +15173,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N194" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="O194" t="n">
+        <v>15.32</v>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -12768,6 +15235,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N195" t="n">
+        <v>-33.69</v>
+      </c>
+      <c r="O195" t="n">
+        <v>0</v>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -12819,6 +15297,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N196" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="O196" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -12870,6 +15359,17 @@
           <t>+12/-3</t>
         </is>
       </c>
+      <c r="N197" t="n">
+        <v>-27.09</v>
+      </c>
+      <c r="O197" t="n">
+        <v>0</v>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -12921,6 +15421,17 @@
           <t>+12/-3</t>
         </is>
       </c>
+      <c r="N198" t="n">
+        <v>-26.52</v>
+      </c>
+      <c r="O198" t="n">
+        <v>0</v>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -12972,6 +15483,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N199" t="n">
+        <v>-39.61</v>
+      </c>
+      <c r="O199" t="n">
+        <v>0</v>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13023,6 +15545,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N200" t="n">
+        <v>-10.98</v>
+      </c>
+      <c r="O200" t="n">
+        <v>0</v>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13074,6 +15607,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N201" t="n">
+        <v>-52.69</v>
+      </c>
+      <c r="O201" t="n">
+        <v>0</v>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -13125,6 +15669,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N202" t="n">
+        <v>-49.37</v>
+      </c>
+      <c r="O202" t="n">
+        <v>0</v>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -13176,6 +15731,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N203" t="n">
+        <v>-15.63</v>
+      </c>
+      <c r="O203" t="n">
+        <v>0</v>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -13227,6 +15793,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N204" t="n">
+        <v>-16.68</v>
+      </c>
+      <c r="O204" t="n">
+        <v>0</v>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -13278,6 +15855,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N205" t="n">
+        <v>-128.62</v>
+      </c>
+      <c r="O205" t="n">
+        <v>0</v>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -13329,6 +15917,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N206" t="n">
+        <v>34.74</v>
+      </c>
+      <c r="O206" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -13380,6 +15979,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N207" t="n">
+        <v>-37.65</v>
+      </c>
+      <c r="O207" t="n">
+        <v>0</v>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -13431,6 +16041,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N208" t="n">
+        <v>18.96</v>
+      </c>
+      <c r="O208" t="n">
+        <v>100</v>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -13482,6 +16103,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N209" t="n">
+        <v>-175.56</v>
+      </c>
+      <c r="O209" t="n">
+        <v>0</v>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -13533,6 +16165,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N210" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="O210" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -13584,6 +16227,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N211" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="O211" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -13635,6 +16289,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N212" t="n">
+        <v>-180.26</v>
+      </c>
+      <c r="O212" t="n">
+        <v>0</v>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -13686,6 +16351,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N213" t="n">
+        <v>22.83</v>
+      </c>
+      <c r="O213" t="n">
+        <v>100</v>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -13737,6 +16413,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N214" t="n">
+        <v>-231.03</v>
+      </c>
+      <c r="O214" t="n">
+        <v>0</v>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -13788,6 +16475,17 @@
           <t>+13/-2</t>
         </is>
       </c>
+      <c r="N215" t="n">
+        <v>24.16</v>
+      </c>
+      <c r="O215" t="n">
+        <v>100</v>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -13839,6 +16537,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N216" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="O216" t="n">
+        <v>100</v>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -13890,6 +16599,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N217" t="n">
+        <v>15.89</v>
+      </c>
+      <c r="O217" t="n">
+        <v>98.52</v>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -13941,6 +16661,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N218" t="n">
+        <v>-177.96</v>
+      </c>
+      <c r="O218" t="n">
+        <v>0</v>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -13992,6 +16723,17 @@
           <t>+0/-15</t>
         </is>
       </c>
+      <c r="N219" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="O219" t="n">
+        <v>31.54</v>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -14043,6 +16785,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N220" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="O220" t="n">
+        <v>74.36</v>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -14094,6 +16847,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N221" t="n">
+        <v>-4.85</v>
+      </c>
+      <c r="O221" t="n">
+        <v>0</v>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -14145,6 +16909,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N222" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="O222" t="n">
+        <v>77.20999999999999</v>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -14196,6 +16971,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N223" t="n">
+        <v>-178.7</v>
+      </c>
+      <c r="O223" t="n">
+        <v>0</v>
+      </c>
+      <c r="P223" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -14247,6 +17033,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N224" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="O224" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -14298,6 +17095,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N225" t="n">
+        <v>-4.85</v>
+      </c>
+      <c r="O225" t="n">
+        <v>0</v>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -14349,6 +17157,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N226" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="O226" t="n">
+        <v>86.81999999999999</v>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -14400,6 +17219,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N227" t="n">
+        <v>18.73</v>
+      </c>
+      <c r="O227" t="n">
+        <v>99.06999999999999</v>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -14451,6 +17281,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N228" t="n">
+        <v>-80.17</v>
+      </c>
+      <c r="O228" t="n">
+        <v>0</v>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -14502,6 +17343,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N229" t="n">
+        <v>-11.47</v>
+      </c>
+      <c r="O229" t="n">
+        <v>0</v>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -14553,6 +17405,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N230" t="n">
+        <v>-40.23</v>
+      </c>
+      <c r="O230" t="n">
+        <v>0</v>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -14604,6 +17467,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N231" t="n">
+        <v>-11.51</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0</v>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -14655,6 +17529,17 @@
           <t>+1/-14</t>
         </is>
       </c>
+      <c r="N232" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="O232" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -14706,6 +17591,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N233" t="n">
+        <v>16.68</v>
+      </c>
+      <c r="O233" t="n">
+        <v>99.17</v>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -14757,6 +17653,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N234" t="n">
+        <v>15.01</v>
+      </c>
+      <c r="O234" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -14808,6 +17715,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N235" t="n">
+        <v>-7.68</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -14859,6 +17777,17 @@
           <t>+14/-1</t>
         </is>
       </c>
+      <c r="N236" t="n">
+        <v>-40.67</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -14910,6 +17839,17 @@
           <t>+15/-0</t>
         </is>
       </c>
+      <c r="N237" t="n">
+        <v>-51.57</v>
+      </c>
+      <c r="O237" t="n">
+        <v>0</v>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -14959,6 +17899,17 @@
       <c r="M238" t="inlineStr">
         <is>
           <t>+15/-0</t>
+        </is>
+      </c>
+      <c r="N238" t="n">
+        <v>-65.68000000000001</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>False</t>
         </is>
       </c>
     </row>

</xml_diff>